<commit_message>
feat(mdg-ai): update AI middleware governance rules, floating composer UI, exact CO volume calculations, and hybrid network support
</commit_message>
<xml_diff>
--- a/PENJUALAN/PART (NOT USE)/INPUT TEST SERIUS.xlsx
+++ b/PENJUALAN/PART (NOT USE)/INPUT TEST SERIUS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\DANIEL\ANTIGRAVITY\MASTER DATA GOVERNANCE\PENJUALAN\PART (NOT USE)\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D04F6F6C-CD8D-4F55-94D7-7D3F3601EB73}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1BD1F925-E086-4004-A43B-98E86F066438}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{FAB06259-2E5B-4DE0-AAE8-F945828C78D8}"/>
   </bookViews>
@@ -133,9 +133,6 @@
     <t>TV= F/B. V. White Beech</t>
   </si>
   <si>
-    <t>ZGW1</t>
-  </si>
-  <si>
     <t>XX</t>
   </si>
   <si>
@@ -236,6 +233,9 @@
   </si>
   <si>
     <t>Storage Location Stock</t>
+  </si>
+  <si>
+    <t>ZRND</t>
   </si>
 </sst>
 </file>
@@ -453,6 +453,15 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -478,15 +487,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="1" fontId="2" fillId="3" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -846,110 +846,110 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:35" x14ac:dyDescent="0.3">
-      <c r="A1" s="26" t="s">
+      <c r="A1" s="17" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="26" t="s">
+      <c r="B1" s="17" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="27" t="s">
+      <c r="C1" s="18" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="27" t="s">
+      <c r="D1" s="18" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="26" t="s">
+      <c r="E1" s="17" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="26" t="s">
+      <c r="F1" s="17" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="26"/>
-      <c r="H1" s="26"/>
-      <c r="I1" s="26"/>
-      <c r="J1" s="26"/>
-      <c r="K1" s="26"/>
+      <c r="G1" s="17"/>
+      <c r="H1" s="17"/>
+      <c r="I1" s="17"/>
+      <c r="J1" s="17"/>
+      <c r="K1" s="17"/>
       <c r="L1" s="1"/>
-      <c r="M1" s="26" t="s">
+      <c r="M1" s="17" t="s">
         <v>3</v>
       </c>
-      <c r="N1" s="26"/>
-      <c r="O1" s="26"/>
-      <c r="P1" s="26" t="s">
+      <c r="N1" s="17"/>
+      <c r="O1" s="17"/>
+      <c r="P1" s="17" t="s">
         <v>6</v>
       </c>
-      <c r="Q1" s="26" t="s">
+      <c r="Q1" s="17" t="s">
         <v>7</v>
       </c>
-      <c r="R1" s="26" t="s">
+      <c r="R1" s="17" t="s">
         <v>8</v>
       </c>
-      <c r="S1" s="26" t="s">
+      <c r="S1" s="17" t="s">
         <v>9</v>
       </c>
-      <c r="T1" s="26" t="s">
+      <c r="T1" s="17" t="s">
         <v>10</v>
       </c>
-      <c r="U1" s="22" t="s">
+      <c r="U1" s="25" t="s">
         <v>11</v>
       </c>
-      <c r="V1" s="23" t="s">
+      <c r="V1" s="26" t="s">
         <v>12</v>
       </c>
-      <c r="W1" s="19" t="s">
+      <c r="W1" s="22" t="s">
         <v>13</v>
       </c>
-      <c r="X1" s="24" t="s">
+      <c r="X1" s="27" t="s">
         <v>14</v>
       </c>
-      <c r="Y1" s="25" t="s">
+      <c r="Y1" s="28" t="s">
         <v>15</v>
       </c>
-      <c r="Z1" s="25" t="s">
+      <c r="Z1" s="28" t="s">
         <v>16</v>
       </c>
-      <c r="AA1" s="19" t="s">
+      <c r="AA1" s="22" t="s">
         <v>17</v>
       </c>
-      <c r="AB1" s="19" t="s">
+      <c r="AB1" s="22" t="s">
         <v>18</v>
       </c>
-      <c r="AC1" s="20" t="s">
+      <c r="AC1" s="23" t="s">
         <v>19</v>
       </c>
-      <c r="AD1" s="20" t="s">
+      <c r="AD1" s="23" t="s">
         <v>20</v>
       </c>
-      <c r="AE1" s="21" t="s">
+      <c r="AE1" s="24" t="s">
         <v>21</v>
       </c>
-      <c r="AF1" s="21"/>
-      <c r="AG1" s="21"/>
-      <c r="AH1" s="21" t="s">
+      <c r="AF1" s="24"/>
+      <c r="AG1" s="24"/>
+      <c r="AH1" s="24" t="s">
         <v>22</v>
       </c>
-      <c r="AI1" s="17" t="s">
+      <c r="AI1" s="20" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="2" spans="1:35" x14ac:dyDescent="0.3">
-      <c r="A2" s="26"/>
-      <c r="B2" s="26"/>
-      <c r="C2" s="28"/>
-      <c r="D2" s="28"/>
-      <c r="E2" s="26"/>
-      <c r="F2" s="18" t="s">
+      <c r="A2" s="17"/>
+      <c r="B2" s="17"/>
+      <c r="C2" s="19"/>
+      <c r="D2" s="19"/>
+      <c r="E2" s="17"/>
+      <c r="F2" s="21" t="s">
         <v>24</v>
       </c>
-      <c r="G2" s="18"/>
-      <c r="H2" s="18" t="s">
+      <c r="G2" s="21"/>
+      <c r="H2" s="21" t="s">
         <v>25</v>
       </c>
-      <c r="I2" s="18"/>
-      <c r="J2" s="18" t="s">
+      <c r="I2" s="21"/>
+      <c r="J2" s="21" t="s">
         <v>26</v>
       </c>
-      <c r="K2" s="18"/>
+      <c r="K2" s="21"/>
       <c r="L2" s="3"/>
       <c r="M2" s="4" t="s">
         <v>24</v>
@@ -960,26 +960,26 @@
       <c r="O2" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="P2" s="26"/>
-      <c r="Q2" s="26"/>
-      <c r="R2" s="26"/>
-      <c r="S2" s="26"/>
-      <c r="T2" s="26"/>
-      <c r="U2" s="22"/>
-      <c r="V2" s="23"/>
-      <c r="W2" s="19"/>
-      <c r="X2" s="24"/>
-      <c r="Y2" s="25"/>
-      <c r="Z2" s="25"/>
-      <c r="AA2" s="19"/>
-      <c r="AB2" s="19"/>
-      <c r="AC2" s="20"/>
-      <c r="AD2" s="20"/>
-      <c r="AE2" s="21"/>
-      <c r="AF2" s="21"/>
-      <c r="AG2" s="21"/>
-      <c r="AH2" s="21"/>
-      <c r="AI2" s="17"/>
+      <c r="P2" s="17"/>
+      <c r="Q2" s="17"/>
+      <c r="R2" s="17"/>
+      <c r="S2" s="17"/>
+      <c r="T2" s="17"/>
+      <c r="U2" s="25"/>
+      <c r="V2" s="26"/>
+      <c r="W2" s="22"/>
+      <c r="X2" s="27"/>
+      <c r="Y2" s="28"/>
+      <c r="Z2" s="28"/>
+      <c r="AA2" s="22"/>
+      <c r="AB2" s="22"/>
+      <c r="AC2" s="23"/>
+      <c r="AD2" s="23"/>
+      <c r="AE2" s="24"/>
+      <c r="AF2" s="24"/>
+      <c r="AG2" s="24"/>
+      <c r="AH2" s="24"/>
+      <c r="AI2" s="20"/>
     </row>
     <row r="3" spans="1:35" x14ac:dyDescent="0.3">
       <c r="A3" s="7">
@@ -1025,10 +1025,10 @@
         <v>31</v>
       </c>
       <c r="U3" s="5" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="V3" s="6" t="s">
-        <v>32</v>
+        <v>66</v>
       </c>
       <c r="W3" s="5"/>
       <c r="X3" s="7"/>
@@ -1058,24 +1058,12 @@
         <v>99999</v>
       </c>
       <c r="AH3" s="9" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="AI3" s="12"/>
     </row>
   </sheetData>
   <mergeCells count="28">
-    <mergeCell ref="T1:T2"/>
-    <mergeCell ref="A1:A2"/>
-    <mergeCell ref="B1:B2"/>
-    <mergeCell ref="C1:C2"/>
-    <mergeCell ref="D1:D2"/>
-    <mergeCell ref="E1:E2"/>
-    <mergeCell ref="F1:K1"/>
-    <mergeCell ref="M1:O1"/>
-    <mergeCell ref="P1:P2"/>
-    <mergeCell ref="Q1:Q2"/>
-    <mergeCell ref="R1:R2"/>
-    <mergeCell ref="S1:S2"/>
     <mergeCell ref="AI1:AI2"/>
     <mergeCell ref="F2:G2"/>
     <mergeCell ref="H2:I2"/>
@@ -1092,6 +1080,18 @@
     <mergeCell ref="X1:X2"/>
     <mergeCell ref="Y1:Y2"/>
     <mergeCell ref="Z1:Z2"/>
+    <mergeCell ref="T1:T2"/>
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="B1:B2"/>
+    <mergeCell ref="C1:C2"/>
+    <mergeCell ref="D1:D2"/>
+    <mergeCell ref="E1:E2"/>
+    <mergeCell ref="F1:K1"/>
+    <mergeCell ref="M1:O1"/>
+    <mergeCell ref="P1:P2"/>
+    <mergeCell ref="Q1:Q2"/>
+    <mergeCell ref="R1:R2"/>
+    <mergeCell ref="S1:S2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1108,228 +1108,228 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B3" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B4" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B5" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B6" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B7" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B8" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B9" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B10" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B11" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B12" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B13" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B14" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B15" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B16" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B17" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B18" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B19" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B20" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B21" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B22" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B23" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B24" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B25" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B26" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B27" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B28" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B29" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
   </sheetData>

</xml_diff>